<commit_message>
SGUX-0003 MOTD and SGUX-0004 LogLevel
</commit_message>
<xml_diff>
--- a/SolidgroundUX devlog.xlsx
+++ b/SolidgroundUX devlog.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Mark\Files\Development\Linux.sh\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Mark\Files\Development\Linux.sh\solidgroundux\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E5DD6E6-316F-4D8F-B821-47072E989873}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C178C3B-8ED3-443E-B9F9-9ED11E8887E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18135" yWindow="3240" windowWidth="48255" windowHeight="31470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="18135" yWindow="480" windowWidth="48255" windowHeight="31470" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Devlog" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -91,6 +91,42 @@
   </si>
   <si>
     <t>-</t>
+  </si>
+  <si>
+    <t>SGUX-0002</t>
+  </si>
+  <si>
+    <t>Install procedure</t>
+  </si>
+  <si>
+    <t>Chicken and egg</t>
+  </si>
+  <si>
+    <t>On first install the sequence of events was murky at best</t>
+  </si>
+  <si>
+    <t>Changed code to ignore reccursive trees</t>
+  </si>
+  <si>
+    <t>Redefined, adapted INSTALL.md and documentation accordingly</t>
+  </si>
+  <si>
+    <t>SGUX-0003</t>
+  </si>
+  <si>
+    <t>MOTD</t>
+  </si>
+  <si>
+    <t>CR</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Add decent framework style motd</t>
+  </si>
+  <si>
+    <t>Adapted 90_solidgroundux</t>
   </si>
 </sst>
 </file>
@@ -442,18 +478,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
     <col min="4" max="4" width="12" style="7" customWidth="1"/>
     <col min="5" max="5" width="5.42578125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="31.42578125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="49.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -516,18 +553,65 @@
       <c r="I2" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="J2" s="1" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="3" spans="1:10">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
+      <c r="A3" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>15</v>
+      </c>
       <c r="D3" s="6"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="1"/>
-      <c r="I3" s="1"/>
-      <c r="J3" s="1"/>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" s="2">
+        <v>46186</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2">
+        <v>46189</v>
+      </c>
+      <c r="H4" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>